<commit_message>
Reporte actualizado automaticamente el 2026-10-16
</commit_message>
<xml_diff>
--- a/Programmes Seguimiento LE_2.xlsx
+++ b/Programmes Seguimiento LE_2.xlsx
@@ -180,7 +180,7 @@
     <t xml:space="preserve">Tv Programs</t>
   </si>
   <si>
-    <t xml:space="preserve">20/08/2026 - 21/08/2026;   24/08/2026 - 28/08/2026;   31/08/2026 - 04/09/2026;   07/09/2026 - 11/09/2026;   14/09/2026 - 18/09/2026;   21/09/2026 - 25/09/2026;   28/09/2026 - 02/10/2026;   05/10/2026 - 09/10/2026;   12/10/2026 - 14/10/2026</t>
+    <t xml:space="preserve">20/08/2026 - 21/08/2026;   24/08/2026 - 28/08/2026;   31/08/2026 - 04/09/2026;   07/09/2026 - 11/09/2026;   14/09/2026 - 18/09/2026;   21/09/2026 - 25/09/2026;   28/09/2026 - 02/10/2026;   05/10/2026 - 09/10/2026;   12/10/2026 - 15/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">National</t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet0.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H602"/>
+  <dimension ref="A1:H617"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="22.86" customWidth="1"/>
@@ -16129,6 +16129,396 @@
       </c>
       <c r="H602" s="5" t="n">
         <v>569.872254</v>
+      </c>
+    </row>
+    <row r="603" spans="1:8" ht="18" customHeight="1">
+      <c r="A603" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B603" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C603" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D603" s="4">
+        <v>0.244560185185185</v>
+      </c>
+      <c r="E603" s="4">
+        <v>0.2896875</v>
+      </c>
+      <c r="F603" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G603" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H603" s="5" t="n">
+        <v>492.833961</v>
+      </c>
+    </row>
+    <row r="604" spans="1:8" ht="18" customHeight="1">
+      <c r="A604" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B604" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C604" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D604" s="4">
+        <v>0.2896875</v>
+      </c>
+      <c r="E604" s="4">
+        <v>0.333483796296296</v>
+      </c>
+      <c r="F604" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G604" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H604" s="5" t="n">
+        <v>932.426538</v>
+      </c>
+    </row>
+    <row r="605" spans="1:8" ht="18" customHeight="1">
+      <c r="A605" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B605" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C605" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D605" s="4">
+        <v>0.333483796296296</v>
+      </c>
+      <c r="E605" s="4">
+        <v>0.375023148148148</v>
+      </c>
+      <c r="F605" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G605" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H605" s="5" t="n">
+        <v>1042.901231</v>
+      </c>
+    </row>
+    <row r="606" spans="1:8" ht="18" customHeight="1">
+      <c r="A606" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B606" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C606" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D606" s="4">
+        <v>0.375023148148148</v>
+      </c>
+      <c r="E606" s="4">
+        <v>0.500023148148148</v>
+      </c>
+      <c r="F606" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G606" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H606" s="5" t="n">
+        <v>1398.719412</v>
+      </c>
+    </row>
+    <row r="607" spans="1:8" ht="18" customHeight="1">
+      <c r="A607" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B607" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C607" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D607" s="4">
+        <v>0.500023148148148</v>
+      </c>
+      <c r="E607" s="4">
+        <v>0.562523148148148</v>
+      </c>
+      <c r="F607" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G607" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H607" s="5" t="n">
+        <v>1605.143061</v>
+      </c>
+    </row>
+    <row r="608" spans="1:8" ht="18" customHeight="1">
+      <c r="A608" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B608" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C608" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D608" s="4">
+        <v>0.562523148148148</v>
+      </c>
+      <c r="E608" s="4">
+        <v>0.604166666666667</v>
+      </c>
+      <c r="F608" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G608" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H608" s="5" t="n">
+        <v>1619.948819</v>
+      </c>
+    </row>
+    <row r="609" spans="1:8" ht="18" customHeight="1">
+      <c r="A609" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B609" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C609" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D609" s="4">
+        <v>0.604166666666667</v>
+      </c>
+      <c r="E609" s="4">
+        <v>0.645833333333333</v>
+      </c>
+      <c r="F609" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G609" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H609" s="5" t="n">
+        <v>1965.079312</v>
+      </c>
+    </row>
+    <row r="610" spans="1:8" ht="18" customHeight="1">
+      <c r="A610" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B610" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C610" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D610" s="4">
+        <v>0.645833333333333</v>
+      </c>
+      <c r="E610" s="4">
+        <v>0.6875</v>
+      </c>
+      <c r="F610" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G610" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H610" s="5" t="n">
+        <v>2507.866226</v>
+      </c>
+    </row>
+    <row r="611" spans="1:8" ht="18" customHeight="1">
+      <c r="A611" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B611" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C611" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D611" s="4">
+        <v>0.6875</v>
+      </c>
+      <c r="E611" s="4">
+        <v>0.770868055555556</v>
+      </c>
+      <c r="F611" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G611" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H611" s="5" t="n">
+        <v>3744.490297</v>
+      </c>
+    </row>
+    <row r="612" spans="1:8" ht="18" customHeight="1">
+      <c r="A612" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B612" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C612" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D612" s="4">
+        <v>0.770868055555556</v>
+      </c>
+      <c r="E612" s="4">
+        <v>0.812534722222222</v>
+      </c>
+      <c r="F612" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G612" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H612" s="5" t="n">
+        <v>3703.570586</v>
+      </c>
+    </row>
+    <row r="613" spans="1:8" ht="18" customHeight="1">
+      <c r="A613" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B613" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C613" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D613" s="4">
+        <v>0.812534722222222</v>
+      </c>
+      <c r="E613" s="4">
+        <v>0.854155092592593</v>
+      </c>
+      <c r="F613" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G613" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H613" s="5" t="n">
+        <v>4467.66627</v>
+      </c>
+    </row>
+    <row r="614" spans="1:8" ht="18" customHeight="1">
+      <c r="A614" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B614" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C614" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D614" s="4">
+        <v>0.854155092592593</v>
+      </c>
+      <c r="E614" s="4">
+        <v>0.895833333333333</v>
+      </c>
+      <c r="F614" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G614" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H614" s="5" t="n">
+        <v>4214.642311</v>
+      </c>
+    </row>
+    <row r="615" spans="1:8" ht="18" customHeight="1">
+      <c r="A615" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B615" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C615" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D615" s="4">
+        <v>0.895833333333333</v>
+      </c>
+      <c r="E615" s="4">
+        <v>0.937546296296296</v>
+      </c>
+      <c r="F615" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G615" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H615" s="5" t="n">
+        <v>3800.638643</v>
+      </c>
+    </row>
+    <row r="616" spans="1:8" ht="18" customHeight="1">
+      <c r="A616" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B616" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C616" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D616" s="4">
+        <v>0.937546296296296</v>
+      </c>
+      <c r="E616" s="4">
+        <v>0.962835648148148</v>
+      </c>
+      <c r="F616" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G616" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H616" s="5" t="n">
+        <v>2062.211122</v>
+      </c>
+    </row>
+    <row r="617" spans="1:8" ht="18" customHeight="1">
+      <c r="A617" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B617" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C617" s="3">
+        <v>46310</v>
+      </c>
+      <c r="D617" s="4">
+        <v>0.962835648148148</v>
+      </c>
+      <c r="E617" s="4">
+        <v>1.00642361111111</v>
+      </c>
+      <c r="F617" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G617" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H617" s="5" t="n">
+        <v>664.19503</v>
       </c>
     </row>
   </sheetData>

</xml_diff>